<commit_message>
feat: add iOS sync script, update UI strings, and improve backend comparison CLI.
</commit_message>
<xml_diff>
--- a/Python/Strings Comparer/ExcelData/customer-app-string.xlsx
+++ b/Python/Strings Comparer/ExcelData/customer-app-string.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1862" uniqueCount="1096">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2453" uniqueCount="1477">
   <si>
     <t>Key</t>
   </si>
@@ -3301,6 +3301,1149 @@
   </si>
   <si>
     <t>Please wait until the admin assigns a route to your request. Once the route is set, you can proceed with the payment, and your booking will be confirmed after payment.</t>
+  </si>
+  <si>
+    <t>button_done</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>button_drop</t>
+  </si>
+  <si>
+    <t>Drop</t>
+  </si>
+  <si>
+    <t>booking_status_dropped</t>
+  </si>
+  <si>
+    <t>Dropped</t>
+  </si>
+  <si>
+    <t>booking_status_finishing_last_trip</t>
+  </si>
+  <si>
+    <t>Driver is finishing last trip before picking you up</t>
+  </si>
+  <si>
+    <t>button_accept_terms_and_continue</t>
+  </si>
+  <si>
+    <t>Accept &amp; Continue</t>
+  </si>
+  <si>
+    <t>button_place_order_with_partial_payment</t>
+  </si>
+  <si>
+    <t>Place order with partial payment</t>
+  </si>
+  <si>
+    <t>button_purchase_subscription</t>
+  </si>
+  <si>
+    <t>Purchase Subscription</t>
+  </si>
+  <si>
+    <t>button_renew</t>
+  </si>
+  <si>
+    <t>Renew</t>
+  </si>
+  <si>
+    <t>button_slot</t>
+  </si>
+  <si>
+    <t>Slot</t>
+  </si>
+  <si>
+    <t>button_upgrade</t>
+  </si>
+  <si>
+    <t>Upgrade</t>
+  </si>
+  <si>
+    <t>button_view_benefits</t>
+  </si>
+  <si>
+    <t>View Benefits</t>
+  </si>
+  <si>
+    <t>button_view_referral_policy</t>
+  </si>
+  <si>
+    <t>View Referral Policy</t>
+  </si>
+  <si>
+    <t>button_yes_sure</t>
+  </si>
+  <si>
+    <t>Yes, Sure</t>
+  </si>
+  <si>
+    <t>description_accepted</t>
+  </si>
+  <si>
+    <t>description_action_subscription</t>
+  </si>
+  <si>
+    <t>Are you sure you want to proceed?</t>
+  </si>
+  <si>
+    <t>description_add_contact_info</t>
+  </si>
+  <si>
+    <t>Add Contact Information</t>
+  </si>
+  <si>
+    <t>description_add_courier_item</t>
+  </si>
+  <si>
+    <t>Add Courier Item</t>
+  </si>
+  <si>
+    <t>description_add_modifier</t>
+  </si>
+  <si>
+    <t>Add Modifier</t>
+  </si>
+  <si>
+    <t>description_add_photo</t>
+  </si>
+  <si>
+    <t>We can get your vehicle details from a photo</t>
+  </si>
+  <si>
+    <t>description_additional_info</t>
+  </si>
+  <si>
+    <t>Additional Info</t>
+  </si>
+  <si>
+    <t>description_apple_pay</t>
+  </si>
+  <si>
+    <t>Apple Pay</t>
+  </si>
+  <si>
+    <t>description_arriving_in_mins_qd</t>
+  </si>
+  <si>
+    <t>Arriving in {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_choose_items</t>
+  </si>
+  <si>
+    <t>Choose Items</t>
+  </si>
+  <si>
+    <t>description_courier</t>
+  </si>
+  <si>
+    <t>Courier</t>
+  </si>
+  <si>
+    <t>description_courier_add</t>
+  </si>
+  <si>
+    <t>description_courier_edit</t>
+  </si>
+  <si>
+    <t>description_courier_modifier</t>
+  </si>
+  <si>
+    <t>Modifier</t>
+  </si>
+  <si>
+    <t>description_courier_pickup_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pickup time - </t>
+  </si>
+  <si>
+    <t>description_courier_timeline_title</t>
+  </si>
+  <si>
+    <t>Order Timeline</t>
+  </si>
+  <si>
+    <t>description_delivery_type</t>
+  </si>
+  <si>
+    <t>Delivery Type</t>
+  </si>
+  <si>
+    <t>description_departure_time</t>
+  </si>
+  <si>
+    <t>Departure Time: {{_UNIT_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_description_award_profit_bonus</t>
+  </si>
+  <si>
+    <t>Award Profit Bonus</t>
+  </si>
+  <si>
+    <t>description_dimension</t>
+  </si>
+  <si>
+    <t>Dimension - {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_doc_expired</t>
+  </si>
+  <si>
+    <t>Expired</t>
+  </si>
+  <si>
+    <t>description_drop_off_items</t>
+  </si>
+  <si>
+    <t>Drop off items</t>
+  </si>
+  <si>
+    <t>description_egg</t>
+  </si>
+  <si>
+    <t>Egg</t>
+  </si>
+  <si>
+    <t>description_estimated_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated delivery time - </t>
+  </si>
+  <si>
+    <t>description_expired</t>
+  </si>
+  <si>
+    <t>Expired!</t>
+  </si>
+  <si>
+    <t>description_expires_soon</t>
+  </si>
+  <si>
+    <t>Expires soon!</t>
+  </si>
+  <si>
+    <t>description_express_delivery</t>
+  </si>
+  <si>
+    <t>Express Delivery</t>
+  </si>
+  <si>
+    <t>description_fav_remove</t>
+  </si>
+  <si>
+    <t>Are you sure you want to remove from favourite</t>
+  </si>
+  <si>
+    <t>description_food_type</t>
+  </si>
+  <si>
+    <t>Food type</t>
+  </si>
+  <si>
+    <t>description_free_trial</t>
+  </si>
+  <si>
+    <t>Free Trial</t>
+  </si>
+  <si>
+    <t>description_hyperpay</t>
+  </si>
+  <si>
+    <t>Hyperpay</t>
+  </si>
+  <si>
+    <t>description_images</t>
+  </si>
+  <si>
+    <t>Images</t>
+  </si>
+  <si>
+    <t>description_inter_city_courier</t>
+  </si>
+  <si>
+    <t>Inter City</t>
+  </si>
+  <si>
+    <t>description_intra_city_courier</t>
+  </si>
+  <si>
+    <t>Intra City</t>
+  </si>
+  <si>
+    <t>description_life_time</t>
+  </si>
+  <si>
+    <t>Life Time</t>
+  </si>
+  <si>
+    <t>description_mercado_pago</t>
+  </si>
+  <si>
+    <t>Mercado Pago</t>
+  </si>
+  <si>
+    <t>description_movers_and_packers</t>
+  </si>
+  <si>
+    <t>Movers</t>
+  </si>
+  <si>
+    <t>description_mpesa</t>
+  </si>
+  <si>
+    <t>Mpesa</t>
+  </si>
+  <si>
+    <t>description_name_courier</t>
+  </si>
+  <si>
+    <t>Name: {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_nestpay</t>
+  </si>
+  <si>
+    <t>NestPay</t>
+  </si>
+  <si>
+    <t>description_no_provider_found</t>
+  </si>
+  <si>
+    <t>We’re sorry, there are no nearby drivers available at the moment. We appreciate your business, and we hope you’ll check back soon!</t>
+  </si>
+  <si>
+    <t>description_non_veg</t>
+  </si>
+  <si>
+    <t>Non Veg</t>
+  </si>
+  <si>
+    <t>description_note</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>description_note_colon_value</t>
+  </si>
+  <si>
+    <t>Note: {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_online_service</t>
+  </si>
+  <si>
+    <t>description_onsite_service</t>
+  </si>
+  <si>
+    <t>On Site Service</t>
+  </si>
+  <si>
+    <t>description_order_receive_date</t>
+  </si>
+  <si>
+    <t>Order Receive Time: {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_otp_sd</t>
+  </si>
+  <si>
+    <t>description_pago</t>
+  </si>
+  <si>
+    <t>Pago</t>
+  </si>
+  <si>
+    <t>description_payment_pending</t>
+  </si>
+  <si>
+    <t>Payment is pending!</t>
+  </si>
+  <si>
+    <t>description_paymob</t>
+  </si>
+  <si>
+    <t>Paymob</t>
+  </si>
+  <si>
+    <t>description_payu</t>
+  </si>
+  <si>
+    <t>PayU</t>
+  </si>
+  <si>
+    <t>description_pending</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>description_phone_courier</t>
+  </si>
+  <si>
+    <t>Phone: {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_pickup_items</t>
+  </si>
+  <si>
+    <t>Pickup items</t>
+  </si>
+  <si>
+    <t>description_plan_basic</t>
+  </si>
+  <si>
+    <t>BASIC</t>
+  </si>
+  <si>
+    <t>description_plan_premium</t>
+  </si>
+  <si>
+    <t>PREMIUM</t>
+  </si>
+  <si>
+    <t>description_plan_professional</t>
+  </si>
+  <si>
+    <t>PROFESSIONAL</t>
+  </si>
+  <si>
+    <t>description_plan_standard</t>
+  </si>
+  <si>
+    <t>STANDARD</t>
+  </si>
+  <si>
+    <t>description_pm</t>
+  </si>
+  <si>
+    <t>PM</t>
+  </si>
+  <si>
+    <t>description_product</t>
+  </si>
+  <si>
+    <t>description_qicard</t>
+  </si>
+  <si>
+    <t>QiCard</t>
+  </si>
+  <si>
+    <t>description_quick_delivery</t>
+  </si>
+  <si>
+    <t>Quick Delivery</t>
+  </si>
+  <si>
+    <t>description_referral_list</t>
+  </si>
+  <si>
+    <t>Referral List</t>
+  </si>
+  <si>
+    <t>description_referral_profit_bonus</t>
+  </si>
+  <si>
+    <t>Referral Profit Bonus</t>
+  </si>
+  <si>
+    <t>description_rejected</t>
+  </si>
+  <si>
+    <t>Rejected</t>
+  </si>
+  <si>
+    <t>description_return_time</t>
+  </si>
+  <si>
+    <t>Return Time: {{_UNIT_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_reviews</t>
+  </si>
+  <si>
+    <t>Reviews</t>
+  </si>
+  <si>
+    <t>description_service_at_home</t>
+  </si>
+  <si>
+    <t>Service At Home</t>
+  </si>
+  <si>
+    <t>description_standard_delivery</t>
+  </si>
+  <si>
+    <t>Standard Delivery</t>
+  </si>
+  <si>
+    <t>description_sure_call_sos</t>
+  </si>
+  <si>
+    <t>Are you sure want to call SOS?</t>
+  </si>
+  <si>
+    <t>description_ticket_cancelled</t>
+  </si>
+  <si>
+    <t>CANCELLED</t>
+  </si>
+  <si>
+    <t>description_ticket_closed</t>
+  </si>
+  <si>
+    <t>description_ticket_open</t>
+  </si>
+  <si>
+    <t>description_ticket_reopen</t>
+  </si>
+  <si>
+    <t>description_timeline_accepted</t>
+  </si>
+  <si>
+    <t>Your request has been accepted</t>
+  </si>
+  <si>
+    <t>description_timeline_arrived_at_destination</t>
+  </si>
+  <si>
+    <t>Deliveryman has arrived at destination</t>
+  </si>
+  <si>
+    <t>description_timeline_arrived_at_pickup</t>
+  </si>
+  <si>
+    <t>Deliveryman has arrived at pickup</t>
+  </si>
+  <si>
+    <t>description_timeline_arrived_at_stop</t>
+  </si>
+  <si>
+    <t>Deliveryman has arrived at stop</t>
+  </si>
+  <si>
+    <t>description_timeline_cancelled</t>
+  </si>
+  <si>
+    <t>Your request has been cancelled</t>
+  </si>
+  <si>
+    <t>description_timeline_dropped</t>
+  </si>
+  <si>
+    <t>Package has been dropped off</t>
+  </si>
+  <si>
+    <t>description_timeline_in_route</t>
+  </si>
+  <si>
+    <t>Deliveryman is on the way</t>
+  </si>
+  <si>
+    <t>description_timeline_picked</t>
+  </si>
+  <si>
+    <t>Package has been picked up</t>
+  </si>
+  <si>
+    <t>description_timeline_requested</t>
+  </si>
+  <si>
+    <t>Your request has been placed</t>
+  </si>
+  <si>
+    <t>description_timeline_started</t>
+  </si>
+  <si>
+    <t>Your delivery has started</t>
+  </si>
+  <si>
+    <t>description_uploaded</t>
+  </si>
+  <si>
+    <t>Uploaded</t>
+  </si>
+  <si>
+    <t>description_value_days</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} days</t>
+  </si>
+  <si>
+    <t>description_value_free_trial</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} free trial days</t>
+  </si>
+  <si>
+    <t>description_value_of_parcel</t>
+  </si>
+  <si>
+    <t>Value of parcel - {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_veg</t>
+  </si>
+  <si>
+    <t>Veg</t>
+  </si>
+  <si>
+    <t>description_vegan</t>
+  </si>
+  <si>
+    <t>Vegan</t>
+  </si>
+  <si>
+    <t>description_vehicle_change_cart_alert</t>
+  </si>
+  <si>
+    <t>You already added service from diffrent vehicle. do you want to clear cart and add for current vehicle?</t>
+  </si>
+  <si>
+    <t>description_vehicle_dimension</t>
+  </si>
+  <si>
+    <t>Dimension {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_vehicle_max_weight_capacity</t>
+  </si>
+  <si>
+    <t>Max weight capacity {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_weight</t>
+  </si>
+  <si>
+    <t>Weight - {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_were_house</t>
+  </si>
+  <si>
+    <t>Were house</t>
+  </si>
+  <si>
+    <t>description_with_in_time</t>
+  </si>
+  <si>
+    <t>Within</t>
+  </si>
+  <si>
+    <t>description_you_saved</t>
+  </si>
+  <si>
+    <t>You Saved {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>description_your_booking_cancel</t>
+  </si>
+  <si>
+    <t>Your booking has been canceled</t>
+  </si>
+  <si>
+    <t>description_your_plan_expires_in_days</t>
+  </si>
+  <si>
+    <t>Your plan expires in {{_VALUE}} days!</t>
+  </si>
+  <si>
+    <t>description_zaincash</t>
+  </si>
+  <si>
+    <t>ZainCash</t>
+  </si>
+  <si>
+    <t>error_document_not_accepted</t>
+  </si>
+  <si>
+    <t>Document not accepted</t>
+  </si>
+  <si>
+    <t>error_each_location_must_have_at_least_one_pickdrop_parcel</t>
+  </si>
+  <si>
+    <t>Each location must have at least one pick/drop parcel</t>
+  </si>
+  <si>
+    <t>error_enter_contact_information_to_each_location</t>
+  </si>
+  <si>
+    <t>Enter contact information to each location</t>
+  </si>
+  <si>
+    <t>error_enter_valid_dropoff_address</t>
+  </si>
+  <si>
+    <t>Enter valid drop-off address</t>
+  </si>
+  <si>
+    <t>error_enter_valid_pickup_address</t>
+  </si>
+  <si>
+    <t>Enter valid pickup address</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_char</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} length must be {{_VALUE1}} characters</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_less_or_equal_char</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} length must be less than or equal to {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_less_or_equal_value</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} must be less than or equal to {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_less_than_char</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} length must be less than {{_VALUE1}} characters</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_less_than_value</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} must be less than {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_more_or_equal_char</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} length must be more than or equal to {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_more_or_equal_value</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} must be more than or equal to {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_more_than_char</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} length must be more than {{_VALUE1}} characters</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_more_than_value</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} must be more than {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_length_must_be_value</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} must be {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_length_must_not_be_char</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} length must not be {{_VALUE1}} characters</t>
+  </si>
+  <si>
+    <t>error_field_length_must_not_be_value</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} must not be {{_VALUE1}}</t>
+  </si>
+  <si>
+    <t>error_field_required</t>
+  </si>
+  <si>
+    <t>{{_VALUE}} is required</t>
+  </si>
+  <si>
+    <t>error_height_max_limit_is</t>
+  </si>
+  <si>
+    <t>Height max limit is {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>error_image_max_limit_is</t>
+  </si>
+  <si>
+    <t>Image max limit is {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>error_length_max_limit_is</t>
+  </si>
+  <si>
+    <t>Length max limit is {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>error_microphone_permission_denied</t>
+  </si>
+  <si>
+    <t>Microphone access is required. Please enable it in Settings.</t>
+  </si>
+  <si>
+    <t>error_parcel_value_max_limit_is</t>
+  </si>
+  <si>
+    <t>Parcel value max limit is {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>error_pickup_location_must_contain_at_least_one_parcel</t>
+  </si>
+  <si>
+    <t>Pickup location must contain at least one parcel</t>
+  </si>
+  <si>
+    <t>error_please_enter_height</t>
+  </si>
+  <si>
+    <t>Please enter height</t>
+  </si>
+  <si>
+    <t>error_please_enter_length</t>
+  </si>
+  <si>
+    <t>Please enter length</t>
+  </si>
+  <si>
+    <t>error_please_enter_title</t>
+  </si>
+  <si>
+    <t>Please enter title</t>
+  </si>
+  <si>
+    <t>error_please_enter_valueOfParcel</t>
+  </si>
+  <si>
+    <t>Please enter valueOfParcel</t>
+  </si>
+  <si>
+    <t>error_please_enter_weight</t>
+  </si>
+  <si>
+    <t>Please enter weight</t>
+  </si>
+  <si>
+    <t>error_please_enter_width</t>
+  </si>
+  <si>
+    <t>Please enter width</t>
+  </si>
+  <si>
+    <t>error_please_select</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plese select </t>
+  </si>
+  <si>
+    <t>error_please_select_category</t>
+  </si>
+  <si>
+    <t>Please select category</t>
+  </si>
+  <si>
+    <t>error_please_select_gender</t>
+  </si>
+  <si>
+    <t>Please select gender</t>
+  </si>
+  <si>
+    <t>error_please_select_modifier</t>
+  </si>
+  <si>
+    <t>Plese select modifier</t>
+  </si>
+  <si>
+    <t>error_please_select_modifier_value_sd</t>
+  </si>
+  <si>
+    <t>Please select {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>error_please_select_subcategory</t>
+  </si>
+  <si>
+    <t>Please select subcategory</t>
+  </si>
+  <si>
+    <t>error_please_select_subscription</t>
+  </si>
+  <si>
+    <t>Please select subscription</t>
+  </si>
+  <si>
+    <t>error_select_vehicle_photo</t>
+  </si>
+  <si>
+    <t>Select vehicle photo</t>
+  </si>
+  <si>
+    <t>error_simulator_not_supported</t>
+  </si>
+  <si>
+    <t>Speech recognition isn't available in the simulator. Please use a real device.</t>
+  </si>
+  <si>
+    <t>error_some_parcels_are_not_assigned_to_any_dropoff</t>
+  </si>
+  <si>
+    <t>Some parcels are not assigned to any drop-off</t>
+  </si>
+  <si>
+    <t>error_speech_permission_denied</t>
+  </si>
+  <si>
+    <t>Speech recognition access is required. Please enable it in Settings.</t>
+  </si>
+  <si>
+    <t>error_speech_permission_undetermined</t>
+  </si>
+  <si>
+    <t>Speech recognition permission has not been set. Please grant access when prompted.</t>
+  </si>
+  <si>
+    <t>error_speech_restricted</t>
+  </si>
+  <si>
+    <t>Speech recognition is restricted on your device. Please check parental controls or device settings.</t>
+  </si>
+  <si>
+    <t>error_speech_unknown</t>
+  </si>
+  <si>
+    <t>Speech recognition is currently unavailable due to an unknown issue. Please try again later.</t>
+  </si>
+  <si>
+    <t>error_vehicle_form_empty</t>
+  </si>
+  <si>
+    <t>Please select all fields</t>
+  </si>
+  <si>
+    <t>error_weight_max_limit_is</t>
+  </si>
+  <si>
+    <t>Weight max limit is {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>error_width_max_limit_is</t>
+  </si>
+  <si>
+    <t>Width max limit is {{_VALUE}}</t>
+  </si>
+  <si>
+    <t>error_you_can_only_select_up_to_options_sd</t>
+  </si>
+  <si>
+    <t>error_you_cant_add_duplicate_address</t>
+  </si>
+  <si>
+    <t>You cant add duplicate address</t>
+  </si>
+  <si>
+    <t>heading_add_information</t>
+  </si>
+  <si>
+    <t>Add required information</t>
+  </si>
+  <si>
+    <t>heading_add_photo</t>
+  </si>
+  <si>
+    <t>Add Photo</t>
+  </si>
+  <si>
+    <t>heading_add_vehicle</t>
+  </si>
+  <si>
+    <t>Add Vehicle</t>
+  </si>
+  <si>
+    <t>heading_clear_cart</t>
+  </si>
+  <si>
+    <t>Clear Cart</t>
+  </si>
+  <si>
+    <t>heading_confirmation</t>
+  </si>
+  <si>
+    <t>Confirmation</t>
+  </si>
+  <si>
+    <t>heading_fix_group_booking</t>
+  </si>
+  <si>
+    <t>Fix Group Bookings</t>
+  </si>
+  <si>
+    <t>heading_gender</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>heading_luggage_capacity_preference</t>
+  </si>
+  <si>
+    <t>Luggage Capacity Preference</t>
+  </si>
+  <si>
+    <t>heading_remove</t>
+  </si>
+  <si>
+    <t>Remove</t>
+  </si>
+  <si>
+    <t>heading_select_gender</t>
+  </si>
+  <si>
+    <t>Select Gender</t>
+  </si>
+  <si>
+    <t>heading_select_return_time</t>
+  </si>
+  <si>
+    <t>Return Time</t>
+  </si>
+  <si>
+    <t>heading_select_slot</t>
+  </si>
+  <si>
+    <t>Select slot</t>
+  </si>
+  <si>
+    <t>heading_selected_payment_option</t>
+  </si>
+  <si>
+    <t>Selected Payment Option</t>
+  </si>
+  <si>
+    <t>heading_selected_rental_ride</t>
+  </si>
+  <si>
+    <t>Selected Rental Ride</t>
+  </si>
+  <si>
+    <t>heading_selected_ride</t>
+  </si>
+  <si>
+    <t>Selected Ride</t>
+  </si>
+  <si>
+    <t>heading_subscription</t>
+  </si>
+  <si>
+    <t>Subscription</t>
+  </si>
+  <si>
+    <t>hint_category</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>hint_courier_title</t>
+  </si>
+  <si>
+    <t>hint_height</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>hint_images</t>
+  </si>
+  <si>
+    <t>hint_length</t>
+  </si>
+  <si>
+    <t>Length</t>
+  </si>
+  <si>
+    <t>hint_license_plate</t>
+  </si>
+  <si>
+    <t>License Plate</t>
+  </si>
+  <si>
+    <t>hint_no_of_parcel</t>
+  </si>
+  <si>
+    <t>No of parcel</t>
+  </si>
+  <si>
+    <t>hint_quantity</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>hint_search_from_phone_contact</t>
+  </si>
+  <si>
+    <t>Search from phone contacts</t>
+  </si>
+  <si>
+    <t>hint_subCategory</t>
+  </si>
+  <si>
+    <t>SubCategory</t>
+  </si>
+  <si>
+    <t>hint_value_of_parcel</t>
+  </si>
+  <si>
+    <t>Value of parcel</t>
+  </si>
+  <si>
+    <t>hint_vehicle_brand</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>hint_vehicle_make</t>
+  </si>
+  <si>
+    <t>Vehicle Make</t>
+  </si>
+  <si>
+    <t>hint_vehicle_year</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>hint_weight</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>hint_width</t>
+  </si>
+  <si>
+    <t>width</t>
+  </si>
+  <si>
+    <t>sub_heading_active_subscription</t>
+  </si>
+  <si>
+    <t>Active Subscription</t>
+  </si>
+  <si>
+    <t>sub_heading_subscription</t>
   </si>
 </sst>
 </file>
@@ -3681,7 +4824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I581"/>
+  <dimension ref="A1:I778"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="10" customWidth="1"/>
@@ -10437,6 +11580,2173 @@
         <v>1095</v>
       </c>
     </row>
+    <row r="582" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A582" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B582" t="s">
+        <v>10</v>
+      </c>
+      <c r="C582" t="s">
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="583" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A583" t="s">
+        <v>1098</v>
+      </c>
+      <c r="B583" t="s">
+        <v>10</v>
+      </c>
+      <c r="C583" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="584" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A584" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B584" t="s">
+        <v>10</v>
+      </c>
+      <c r="C584" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="585" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A585" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B585" t="s">
+        <v>10</v>
+      </c>
+      <c r="C585" t="s">
+        <v>1103</v>
+      </c>
+    </row>
+    <row r="586" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A586" t="s">
+        <v>1104</v>
+      </c>
+      <c r="B586" t="s">
+        <v>10</v>
+      </c>
+      <c r="C586" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="587" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A587" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B587" t="s">
+        <v>10</v>
+      </c>
+      <c r="C587" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="588" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A588" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B588" t="s">
+        <v>10</v>
+      </c>
+      <c r="C588" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="589" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A589" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B589" t="s">
+        <v>10</v>
+      </c>
+      <c r="C589" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="590" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A590" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B590" t="s">
+        <v>10</v>
+      </c>
+      <c r="C590" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="591" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A591" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B591" t="s">
+        <v>10</v>
+      </c>
+      <c r="C591" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="592" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A592" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B592" t="s">
+        <v>10</v>
+      </c>
+      <c r="C592" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="593" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A593" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B593" t="s">
+        <v>10</v>
+      </c>
+      <c r="C593" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="594" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A594" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B594" t="s">
+        <v>10</v>
+      </c>
+      <c r="C594" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="595" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A595" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B595" t="s">
+        <v>10</v>
+      </c>
+      <c r="C595" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="596" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A596" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B596" t="s">
+        <v>10</v>
+      </c>
+      <c r="C596" t="s">
+        <v>1124</v>
+      </c>
+    </row>
+    <row r="597" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A597" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B597" t="s">
+        <v>10</v>
+      </c>
+      <c r="C597" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="598" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A598" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B598" t="s">
+        <v>10</v>
+      </c>
+      <c r="C598" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="599" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A599" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B599" t="s">
+        <v>10</v>
+      </c>
+      <c r="C599" t="s">
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="600" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A600" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B600" t="s">
+        <v>10</v>
+      </c>
+      <c r="C600" t="s">
+        <v>1132</v>
+      </c>
+    </row>
+    <row r="601" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A601" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B601" t="s">
+        <v>10</v>
+      </c>
+      <c r="C601" t="s">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="602" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A602" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B602" t="s">
+        <v>10</v>
+      </c>
+      <c r="C602" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="603" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A603" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B603" t="s">
+        <v>10</v>
+      </c>
+      <c r="C603" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="604" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A604" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B604" t="s">
+        <v>10</v>
+      </c>
+      <c r="C604" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="605" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A605" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B605" t="s">
+        <v>10</v>
+      </c>
+      <c r="C605" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="606" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A606" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B606" t="s">
+        <v>10</v>
+      </c>
+      <c r="C606" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="607" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A607" t="s">
+        <v>1144</v>
+      </c>
+      <c r="B607" t="s">
+        <v>10</v>
+      </c>
+      <c r="C607" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="608" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A608" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B608" t="s">
+        <v>10</v>
+      </c>
+      <c r="C608" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="609" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A609" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B609" t="s">
+        <v>10</v>
+      </c>
+      <c r="C609" t="s">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="610" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A610" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B610" t="s">
+        <v>10</v>
+      </c>
+      <c r="C610" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="611" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A611" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B611" t="s">
+        <v>10</v>
+      </c>
+      <c r="C611" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="612" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A612" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B612" t="s">
+        <v>10</v>
+      </c>
+      <c r="C612" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="613" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A613" t="s">
+        <v>1155</v>
+      </c>
+      <c r="B613" t="s">
+        <v>10</v>
+      </c>
+      <c r="C613" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="614" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A614" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B614" t="s">
+        <v>10</v>
+      </c>
+      <c r="C614" t="s">
+        <v>1158</v>
+      </c>
+    </row>
+    <row r="615" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A615" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B615" t="s">
+        <v>10</v>
+      </c>
+      <c r="C615" t="s">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="616" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A616" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B616" t="s">
+        <v>10</v>
+      </c>
+      <c r="C616" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A617" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B617" t="s">
+        <v>10</v>
+      </c>
+      <c r="C617" t="s">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="618" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A618" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B618" t="s">
+        <v>10</v>
+      </c>
+      <c r="C618" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="619" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A619" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B619" t="s">
+        <v>10</v>
+      </c>
+      <c r="C619" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="620" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A620" t="s">
+        <v>1169</v>
+      </c>
+      <c r="B620" t="s">
+        <v>10</v>
+      </c>
+      <c r="C620" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="621" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A621" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B621" t="s">
+        <v>10</v>
+      </c>
+      <c r="C621" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="622" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A622" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B622" t="s">
+        <v>10</v>
+      </c>
+      <c r="C622" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="623" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A623" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B623" t="s">
+        <v>10</v>
+      </c>
+      <c r="C623" t="s">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="624" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A624" t="s">
+        <v>1177</v>
+      </c>
+      <c r="B624" t="s">
+        <v>10</v>
+      </c>
+      <c r="C624" t="s">
+        <v>1178</v>
+      </c>
+    </row>
+    <row r="625" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A625" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B625" t="s">
+        <v>10</v>
+      </c>
+      <c r="C625" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="626" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A626" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B626" t="s">
+        <v>10</v>
+      </c>
+      <c r="C626" t="s">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="627" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A627" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B627" t="s">
+        <v>10</v>
+      </c>
+      <c r="C627" t="s">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="628" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A628" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B628" t="s">
+        <v>10</v>
+      </c>
+      <c r="C628" t="s">
+        <v>1186</v>
+      </c>
+    </row>
+    <row r="629" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A629" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B629" t="s">
+        <v>10</v>
+      </c>
+      <c r="C629" t="s">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="630" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A630" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B630" t="s">
+        <v>10</v>
+      </c>
+      <c r="C630" t="s">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="631" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A631" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B631" t="s">
+        <v>10</v>
+      </c>
+      <c r="C631" t="s">
+        <v>1192</v>
+      </c>
+    </row>
+    <row r="632" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A632" t="s">
+        <v>1193</v>
+      </c>
+      <c r="B632" t="s">
+        <v>10</v>
+      </c>
+      <c r="C632" t="s">
+        <v>1194</v>
+      </c>
+    </row>
+    <row r="633" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A633" t="s">
+        <v>1195</v>
+      </c>
+      <c r="B633" t="s">
+        <v>10</v>
+      </c>
+      <c r="C633" t="s">
+        <v>1196</v>
+      </c>
+    </row>
+    <row r="634" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A634" t="s">
+        <v>1197</v>
+      </c>
+      <c r="B634" t="s">
+        <v>10</v>
+      </c>
+      <c r="C634" t="s">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="635" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A635" t="s">
+        <v>1199</v>
+      </c>
+      <c r="B635" t="s">
+        <v>10</v>
+      </c>
+      <c r="C635" t="s">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="636" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A636" t="s">
+        <v>1201</v>
+      </c>
+      <c r="B636" t="s">
+        <v>10</v>
+      </c>
+      <c r="C636" t="s">
+        <v>1202</v>
+      </c>
+    </row>
+    <row r="637" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A637" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B637" t="s">
+        <v>10</v>
+      </c>
+      <c r="C637" t="s">
+        <v>1204</v>
+      </c>
+    </row>
+    <row r="638" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A638" t="s">
+        <v>1205</v>
+      </c>
+      <c r="B638" t="s">
+        <v>10</v>
+      </c>
+      <c r="C638" t="s">
+        <v>1206</v>
+      </c>
+    </row>
+    <row r="639" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A639" t="s">
+        <v>1207</v>
+      </c>
+      <c r="B639" t="s">
+        <v>10</v>
+      </c>
+      <c r="C639" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="640" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A640" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B640" t="s">
+        <v>10</v>
+      </c>
+      <c r="C640" t="s">
+        <v>1209</v>
+      </c>
+    </row>
+    <row r="641" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A641" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B641" t="s">
+        <v>10</v>
+      </c>
+      <c r="C641" t="s">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="642" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A642" t="s">
+        <v>1212</v>
+      </c>
+      <c r="B642" t="s">
+        <v>10</v>
+      </c>
+      <c r="C642" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="643" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A643" t="s">
+        <v>1213</v>
+      </c>
+      <c r="B643" t="s">
+        <v>10</v>
+      </c>
+      <c r="C643" t="s">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="644" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A644" t="s">
+        <v>1215</v>
+      </c>
+      <c r="B644" t="s">
+        <v>10</v>
+      </c>
+      <c r="C644" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="645" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A645" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B645" t="s">
+        <v>10</v>
+      </c>
+      <c r="C645" t="s">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="646" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A646" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B646" t="s">
+        <v>10</v>
+      </c>
+      <c r="C646" t="s">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="647" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A647" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B647" t="s">
+        <v>10</v>
+      </c>
+      <c r="C647" t="s">
+        <v>1222</v>
+      </c>
+    </row>
+    <row r="648" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A648" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B648" t="s">
+        <v>10</v>
+      </c>
+      <c r="C648" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="649" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A649" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B649" t="s">
+        <v>10</v>
+      </c>
+      <c r="C649" t="s">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="650" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A650" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B650" t="s">
+        <v>10</v>
+      </c>
+      <c r="C650" t="s">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="651" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A651" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B651" t="s">
+        <v>10</v>
+      </c>
+      <c r="C651" t="s">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="652" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A652" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B652" t="s">
+        <v>10</v>
+      </c>
+      <c r="C652" t="s">
+        <v>1232</v>
+      </c>
+    </row>
+    <row r="653" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A653" t="s">
+        <v>1233</v>
+      </c>
+      <c r="B653" t="s">
+        <v>10</v>
+      </c>
+      <c r="C653" t="s">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="654" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A654" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B654" t="s">
+        <v>10</v>
+      </c>
+      <c r="C654" t="s">
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="655" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A655" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B655" t="s">
+        <v>10</v>
+      </c>
+      <c r="C655" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="656" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A656" t="s">
+        <v>1238</v>
+      </c>
+      <c r="B656" t="s">
+        <v>10</v>
+      </c>
+      <c r="C656" t="s">
+        <v>1239</v>
+      </c>
+    </row>
+    <row r="657" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A657" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B657" t="s">
+        <v>10</v>
+      </c>
+      <c r="C657" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="658" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A658" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B658" t="s">
+        <v>10</v>
+      </c>
+      <c r="C658" t="s">
+        <v>1243</v>
+      </c>
+    </row>
+    <row r="659" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A659" t="s">
+        <v>1244</v>
+      </c>
+      <c r="B659" t="s">
+        <v>10</v>
+      </c>
+      <c r="C659" t="s">
+        <v>1245</v>
+      </c>
+    </row>
+    <row r="660" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A660" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B660" t="s">
+        <v>10</v>
+      </c>
+      <c r="C660" t="s">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="661" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A661" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B661" t="s">
+        <v>10</v>
+      </c>
+      <c r="C661" t="s">
+        <v>1249</v>
+      </c>
+    </row>
+    <row r="662" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A662" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B662" t="s">
+        <v>10</v>
+      </c>
+      <c r="C662" t="s">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="663" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A663" t="s">
+        <v>1252</v>
+      </c>
+      <c r="B663" t="s">
+        <v>10</v>
+      </c>
+      <c r="C663" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="664" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A664" t="s">
+        <v>1254</v>
+      </c>
+      <c r="B664" t="s">
+        <v>10</v>
+      </c>
+      <c r="C664" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="665" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A665" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B665" t="s">
+        <v>10</v>
+      </c>
+      <c r="C665" t="s">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="666" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A666" t="s">
+        <v>1258</v>
+      </c>
+      <c r="B666" t="s">
+        <v>10</v>
+      </c>
+      <c r="C666" t="s">
+        <v>1259</v>
+      </c>
+    </row>
+    <row r="667" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A667" t="s">
+        <v>1260</v>
+      </c>
+      <c r="B667" t="s">
+        <v>10</v>
+      </c>
+      <c r="C667" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="668" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A668" t="s">
+        <v>1261</v>
+      </c>
+      <c r="B668" t="s">
+        <v>10</v>
+      </c>
+      <c r="C668" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="669" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A669" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B669" t="s">
+        <v>10</v>
+      </c>
+      <c r="C669" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="670" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A670" t="s">
+        <v>1263</v>
+      </c>
+      <c r="B670" t="s">
+        <v>10</v>
+      </c>
+      <c r="C670" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="671" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A671" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B671" t="s">
+        <v>10</v>
+      </c>
+      <c r="C671" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="672" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A672" t="s">
+        <v>1267</v>
+      </c>
+      <c r="B672" t="s">
+        <v>10</v>
+      </c>
+      <c r="C672" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="673" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A673" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B673" t="s">
+        <v>10</v>
+      </c>
+      <c r="C673" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="674" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A674" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B674" t="s">
+        <v>10</v>
+      </c>
+      <c r="C674" t="s">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="675" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A675" t="s">
+        <v>1273</v>
+      </c>
+      <c r="B675" t="s">
+        <v>10</v>
+      </c>
+      <c r="C675" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="676" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A676" t="s">
+        <v>1275</v>
+      </c>
+      <c r="B676" t="s">
+        <v>10</v>
+      </c>
+      <c r="C676" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="677" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A677" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B677" t="s">
+        <v>10</v>
+      </c>
+      <c r="C677" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="678" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A678" t="s">
+        <v>1279</v>
+      </c>
+      <c r="B678" t="s">
+        <v>10</v>
+      </c>
+      <c r="C678" t="s">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="679" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A679" t="s">
+        <v>1281</v>
+      </c>
+      <c r="B679" t="s">
+        <v>10</v>
+      </c>
+      <c r="C679" t="s">
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="680" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A680" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B680" t="s">
+        <v>10</v>
+      </c>
+      <c r="C680" t="s">
+        <v>1284</v>
+      </c>
+    </row>
+    <row r="681" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A681" t="s">
+        <v>1285</v>
+      </c>
+      <c r="B681" t="s">
+        <v>10</v>
+      </c>
+      <c r="C681" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="682" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A682" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B682" t="s">
+        <v>10</v>
+      </c>
+      <c r="C682" t="s">
+        <v>1288</v>
+      </c>
+    </row>
+    <row r="683" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A683" t="s">
+        <v>1289</v>
+      </c>
+      <c r="B683" t="s">
+        <v>10</v>
+      </c>
+      <c r="C683" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="684" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A684" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B684" t="s">
+        <v>10</v>
+      </c>
+      <c r="C684" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="685" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A685" t="s">
+        <v>1293</v>
+      </c>
+      <c r="B685" t="s">
+        <v>10</v>
+      </c>
+      <c r="C685" t="s">
+        <v>1294</v>
+      </c>
+    </row>
+    <row r="686" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A686" t="s">
+        <v>1295</v>
+      </c>
+      <c r="B686" t="s">
+        <v>10</v>
+      </c>
+      <c r="C686" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="687" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A687" t="s">
+        <v>1297</v>
+      </c>
+      <c r="B687" t="s">
+        <v>10</v>
+      </c>
+      <c r="C687" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="688" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A688" t="s">
+        <v>1299</v>
+      </c>
+      <c r="B688" t="s">
+        <v>10</v>
+      </c>
+      <c r="C688" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="689" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A689" t="s">
+        <v>1301</v>
+      </c>
+      <c r="B689" t="s">
+        <v>10</v>
+      </c>
+      <c r="C689" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="690" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A690" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B690" t="s">
+        <v>10</v>
+      </c>
+      <c r="C690" t="s">
+        <v>1304</v>
+      </c>
+    </row>
+    <row r="691" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A691" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B691" t="s">
+        <v>10</v>
+      </c>
+      <c r="C691" t="s">
+        <v>1306</v>
+      </c>
+    </row>
+    <row r="692" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A692" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B692" t="s">
+        <v>10</v>
+      </c>
+      <c r="C692" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="693" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A693" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B693" t="s">
+        <v>10</v>
+      </c>
+      <c r="C693" t="s">
+        <v>1310</v>
+      </c>
+    </row>
+    <row r="694" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A694" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B694" t="s">
+        <v>10</v>
+      </c>
+      <c r="C694" t="s">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="695" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A695" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B695" t="s">
+        <v>10</v>
+      </c>
+      <c r="C695" t="s">
+        <v>1314</v>
+      </c>
+    </row>
+    <row r="696" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A696" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B696" t="s">
+        <v>10</v>
+      </c>
+      <c r="C696" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="697" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A697" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B697" t="s">
+        <v>10</v>
+      </c>
+      <c r="C697" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="698" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A698" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B698" t="s">
+        <v>10</v>
+      </c>
+      <c r="C698" t="s">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="699" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A699" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B699" t="s">
+        <v>10</v>
+      </c>
+      <c r="C699" t="s">
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="700" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A700" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B700" t="s">
+        <v>10</v>
+      </c>
+      <c r="C700" t="s">
+        <v>1324</v>
+      </c>
+    </row>
+    <row r="701" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A701" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B701" t="s">
+        <v>10</v>
+      </c>
+      <c r="C701" t="s">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="702" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A702" t="s">
+        <v>1327</v>
+      </c>
+      <c r="B702" t="s">
+        <v>10</v>
+      </c>
+      <c r="C702" t="s">
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="703" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A703" t="s">
+        <v>1329</v>
+      </c>
+      <c r="B703" t="s">
+        <v>10</v>
+      </c>
+      <c r="C703" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="704" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A704" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B704" t="s">
+        <v>10</v>
+      </c>
+      <c r="C704" t="s">
+        <v>1332</v>
+      </c>
+    </row>
+    <row r="705" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A705" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B705" t="s">
+        <v>10</v>
+      </c>
+      <c r="C705" t="s">
+        <v>1334</v>
+      </c>
+    </row>
+    <row r="706" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A706" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B706" t="s">
+        <v>10</v>
+      </c>
+      <c r="C706" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="707" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A707" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B707" t="s">
+        <v>10</v>
+      </c>
+      <c r="C707" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="708" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A708" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B708" t="s">
+        <v>10</v>
+      </c>
+      <c r="C708" t="s">
+        <v>1340</v>
+      </c>
+    </row>
+    <row r="709" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A709" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B709" t="s">
+        <v>10</v>
+      </c>
+      <c r="C709" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="710" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A710" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B710" t="s">
+        <v>10</v>
+      </c>
+      <c r="C710" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="711" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A711" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B711" t="s">
+        <v>10</v>
+      </c>
+      <c r="C711" t="s">
+        <v>1346</v>
+      </c>
+    </row>
+    <row r="712" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A712" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B712" t="s">
+        <v>10</v>
+      </c>
+      <c r="C712" t="s">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="713" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A713" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B713" t="s">
+        <v>10</v>
+      </c>
+      <c r="C713" t="s">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="714" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A714" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B714" t="s">
+        <v>10</v>
+      </c>
+      <c r="C714" t="s">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="715" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A715" t="s">
+        <v>1353</v>
+      </c>
+      <c r="B715" t="s">
+        <v>10</v>
+      </c>
+      <c r="C715" t="s">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="716" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A716" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B716" t="s">
+        <v>10</v>
+      </c>
+      <c r="C716" t="s">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="717" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A717" t="s">
+        <v>1357</v>
+      </c>
+      <c r="B717" t="s">
+        <v>10</v>
+      </c>
+      <c r="C717" t="s">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="718" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A718" t="s">
+        <v>1359</v>
+      </c>
+      <c r="B718" t="s">
+        <v>10</v>
+      </c>
+      <c r="C718" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="719" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A719" t="s">
+        <v>1361</v>
+      </c>
+      <c r="B719" t="s">
+        <v>10</v>
+      </c>
+      <c r="C719" t="s">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="720" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A720" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B720" t="s">
+        <v>10</v>
+      </c>
+      <c r="C720" t="s">
+        <v>1364</v>
+      </c>
+    </row>
+    <row r="721" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A721" t="s">
+        <v>1365</v>
+      </c>
+      <c r="B721" t="s">
+        <v>10</v>
+      </c>
+      <c r="C721" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="722" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A722" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B722" t="s">
+        <v>10</v>
+      </c>
+      <c r="C722" t="s">
+        <v>1368</v>
+      </c>
+    </row>
+    <row r="723" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A723" t="s">
+        <v>1369</v>
+      </c>
+      <c r="B723" t="s">
+        <v>10</v>
+      </c>
+      <c r="C723" t="s">
+        <v>1370</v>
+      </c>
+    </row>
+    <row r="724" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A724" t="s">
+        <v>1371</v>
+      </c>
+      <c r="B724" t="s">
+        <v>10</v>
+      </c>
+      <c r="C724" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="725" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A725" t="s">
+        <v>1373</v>
+      </c>
+      <c r="B725" t="s">
+        <v>10</v>
+      </c>
+      <c r="C725" t="s">
+        <v>1374</v>
+      </c>
+    </row>
+    <row r="726" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A726" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B726" t="s">
+        <v>10</v>
+      </c>
+      <c r="C726" t="s">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="727" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A727" t="s">
+        <v>1377</v>
+      </c>
+      <c r="B727" t="s">
+        <v>10</v>
+      </c>
+      <c r="C727" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="728" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A728" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B728" t="s">
+        <v>10</v>
+      </c>
+      <c r="C728" t="s">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="729" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A729" t="s">
+        <v>1381</v>
+      </c>
+      <c r="B729" t="s">
+        <v>10</v>
+      </c>
+      <c r="C729" t="s">
+        <v>1382</v>
+      </c>
+    </row>
+    <row r="730" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A730" t="s">
+        <v>1383</v>
+      </c>
+      <c r="B730" t="s">
+        <v>10</v>
+      </c>
+      <c r="C730" t="s">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="731" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A731" t="s">
+        <v>1385</v>
+      </c>
+      <c r="B731" t="s">
+        <v>10</v>
+      </c>
+      <c r="C731" t="s">
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="732" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A732" t="s">
+        <v>1387</v>
+      </c>
+      <c r="B732" t="s">
+        <v>10</v>
+      </c>
+      <c r="C732" t="s">
+        <v>1388</v>
+      </c>
+    </row>
+    <row r="733" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A733" t="s">
+        <v>1389</v>
+      </c>
+      <c r="B733" t="s">
+        <v>10</v>
+      </c>
+      <c r="C733" t="s">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="734" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A734" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B734" t="s">
+        <v>10</v>
+      </c>
+      <c r="C734" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="735" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A735" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B735" t="s">
+        <v>10</v>
+      </c>
+      <c r="C735" t="s">
+        <v>1394</v>
+      </c>
+    </row>
+    <row r="736" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A736" t="s">
+        <v>1395</v>
+      </c>
+      <c r="B736" t="s">
+        <v>10</v>
+      </c>
+      <c r="C736" t="s">
+        <v>1396</v>
+      </c>
+    </row>
+    <row r="737" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A737" t="s">
+        <v>1397</v>
+      </c>
+      <c r="B737" t="s">
+        <v>10</v>
+      </c>
+      <c r="C737" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="738" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A738" t="s">
+        <v>1399</v>
+      </c>
+      <c r="B738" t="s">
+        <v>10</v>
+      </c>
+      <c r="C738" t="s">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="739" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A739" t="s">
+        <v>1401</v>
+      </c>
+      <c r="B739" t="s">
+        <v>10</v>
+      </c>
+      <c r="C739" t="s">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="740" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A740" t="s">
+        <v>1403</v>
+      </c>
+      <c r="B740" t="s">
+        <v>10</v>
+      </c>
+      <c r="C740" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="741" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A741" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B741" t="s">
+        <v>10</v>
+      </c>
+      <c r="C741" t="s">
+        <v>1406</v>
+      </c>
+    </row>
+    <row r="742" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A742" t="s">
+        <v>1407</v>
+      </c>
+      <c r="B742" t="s">
+        <v>10</v>
+      </c>
+      <c r="C742" t="s">
+        <v>1408</v>
+      </c>
+    </row>
+    <row r="743" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A743" t="s">
+        <v>1409</v>
+      </c>
+      <c r="B743" t="s">
+        <v>10</v>
+      </c>
+      <c r="C743" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="744" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A744" t="s">
+        <v>1410</v>
+      </c>
+      <c r="B744" t="s">
+        <v>10</v>
+      </c>
+      <c r="C744" t="s">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="745" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A745" t="s">
+        <v>1412</v>
+      </c>
+      <c r="B745" t="s">
+        <v>10</v>
+      </c>
+      <c r="C745" t="s">
+        <v>1413</v>
+      </c>
+    </row>
+    <row r="746" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A746" t="s">
+        <v>1414</v>
+      </c>
+      <c r="B746" t="s">
+        <v>10</v>
+      </c>
+      <c r="C746" t="s">
+        <v>1415</v>
+      </c>
+    </row>
+    <row r="747" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A747" t="s">
+        <v>1416</v>
+      </c>
+      <c r="B747" t="s">
+        <v>10</v>
+      </c>
+      <c r="C747" t="s">
+        <v>1417</v>
+      </c>
+    </row>
+    <row r="748" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A748" t="s">
+        <v>1418</v>
+      </c>
+      <c r="B748" t="s">
+        <v>10</v>
+      </c>
+      <c r="C748" t="s">
+        <v>1419</v>
+      </c>
+    </row>
+    <row r="749" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A749" t="s">
+        <v>1420</v>
+      </c>
+      <c r="B749" t="s">
+        <v>10</v>
+      </c>
+      <c r="C749" t="s">
+        <v>1421</v>
+      </c>
+    </row>
+    <row r="750" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A750" t="s">
+        <v>1422</v>
+      </c>
+      <c r="B750" t="s">
+        <v>10</v>
+      </c>
+      <c r="C750" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="751" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A751" t="s">
+        <v>1424</v>
+      </c>
+      <c r="B751" t="s">
+        <v>10</v>
+      </c>
+      <c r="C751" t="s">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="752" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A752" t="s">
+        <v>1426</v>
+      </c>
+      <c r="B752" t="s">
+        <v>10</v>
+      </c>
+      <c r="C752" t="s">
+        <v>1427</v>
+      </c>
+    </row>
+    <row r="753" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A753" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B753" t="s">
+        <v>10</v>
+      </c>
+      <c r="C753" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="754" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A754" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B754" t="s">
+        <v>10</v>
+      </c>
+      <c r="C754" t="s">
+        <v>1431</v>
+      </c>
+    </row>
+    <row r="755" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A755" t="s">
+        <v>1432</v>
+      </c>
+      <c r="B755" t="s">
+        <v>10</v>
+      </c>
+      <c r="C755" t="s">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="756" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A756" t="s">
+        <v>1434</v>
+      </c>
+      <c r="B756" t="s">
+        <v>10</v>
+      </c>
+      <c r="C756" t="s">
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="757" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A757" t="s">
+        <v>1436</v>
+      </c>
+      <c r="B757" t="s">
+        <v>10</v>
+      </c>
+      <c r="C757" t="s">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="758" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A758" t="s">
+        <v>1438</v>
+      </c>
+      <c r="B758" t="s">
+        <v>10</v>
+      </c>
+      <c r="C758" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="759" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A759" t="s">
+        <v>1440</v>
+      </c>
+      <c r="B759" t="s">
+        <v>10</v>
+      </c>
+      <c r="C759" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="760" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A760" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B760" t="s">
+        <v>10</v>
+      </c>
+      <c r="C760" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="761" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A761" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B761" t="s">
+        <v>10</v>
+      </c>
+      <c r="C761" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="762" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A762" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B762" t="s">
+        <v>10</v>
+      </c>
+      <c r="C762" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="763" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A763" t="s">
+        <v>1447</v>
+      </c>
+      <c r="B763" t="s">
+        <v>10</v>
+      </c>
+      <c r="C763" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="764" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A764" t="s">
+        <v>1449</v>
+      </c>
+      <c r="B764" t="s">
+        <v>10</v>
+      </c>
+      <c r="C764" t="s">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="765" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A765" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B765" t="s">
+        <v>10</v>
+      </c>
+      <c r="C765" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="766" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A766" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B766" t="s">
+        <v>10</v>
+      </c>
+      <c r="C766" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="767" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A767" t="s">
+        <v>1454</v>
+      </c>
+      <c r="B767" t="s">
+        <v>10</v>
+      </c>
+      <c r="C767" t="s">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="768" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A768" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B768" t="s">
+        <v>10</v>
+      </c>
+      <c r="C768" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="769" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A769" t="s">
+        <v>1458</v>
+      </c>
+      <c r="B769" t="s">
+        <v>10</v>
+      </c>
+      <c r="C769" t="s">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="770" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A770" t="s">
+        <v>1460</v>
+      </c>
+      <c r="B770" t="s">
+        <v>10</v>
+      </c>
+      <c r="C770" t="s">
+        <v>1461</v>
+      </c>
+    </row>
+    <row r="771" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A771" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B771" t="s">
+        <v>10</v>
+      </c>
+      <c r="C771" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="772" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A772" t="s">
+        <v>1464</v>
+      </c>
+      <c r="B772" t="s">
+        <v>10</v>
+      </c>
+      <c r="C772" t="s">
+        <v>1465</v>
+      </c>
+    </row>
+    <row r="773" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A773" t="s">
+        <v>1466</v>
+      </c>
+      <c r="B773" t="s">
+        <v>10</v>
+      </c>
+      <c r="C773" t="s">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="774" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A774" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B774" t="s">
+        <v>10</v>
+      </c>
+      <c r="C774" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="775" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A775" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B775" t="s">
+        <v>10</v>
+      </c>
+      <c r="C775" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="776" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A776" t="s">
+        <v>1472</v>
+      </c>
+      <c r="B776" t="s">
+        <v>10</v>
+      </c>
+      <c r="C776" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="777" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A777" t="s">
+        <v>1474</v>
+      </c>
+      <c r="B777" t="s">
+        <v>10</v>
+      </c>
+      <c r="C777" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="778" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A778" t="s">
+        <v>1476</v>
+      </c>
+      <c r="B778" t="s">
+        <v>10</v>
+      </c>
+      <c r="C778" t="s">
+        <v>1443</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>